<commit_message>
Complete Days 1-3 deliverables
</commit_message>
<xml_diff>
--- a/output/peer_comparison.xlsx
+++ b/output/peer_comparison.xlsx
@@ -36,12 +36,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD966"/>
+        <bgColor rgb="00FFD966"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -74,11 +80,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -607,26 +614,24 @@
         <v>6558</v>
       </c>
       <c r="O2" t="n">
-        <v>7.72</v>
+        <v>15.22</v>
       </c>
       <c r="P2" t="n">
-        <v>7.39</v>
+        <v>10.99</v>
       </c>
       <c r="Q2" t="n">
-        <v>7.7</v>
+        <v>11.86</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
           <t>Automobiles</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S2" t="n">
+        <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>32.353</v>
+        <v>34.573</v>
       </c>
       <c r="U2" t="n">
         <v>1</v>
@@ -638,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HEROMOTOCO</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -647,74 +652,72 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>10.31</v>
+        <v>24.97</v>
       </c>
       <c r="D3" t="n">
-        <v>86.13</v>
+        <v>26.17</v>
       </c>
       <c r="E3" t="n">
-        <v>21.14</v>
+        <v>22.17</v>
       </c>
       <c r="F3" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="G3" t="n">
-        <v>37.19</v>
+        <v>117</v>
       </c>
       <c r="H3" t="n">
-        <v>1.44</v>
+        <v>0.72</v>
       </c>
       <c r="I3" t="n">
-        <v>6751</v>
+        <v>6558</v>
       </c>
       <c r="J3" t="n">
-        <v>1828</v>
+        <v>2834</v>
       </c>
       <c r="K3" t="n">
-        <v>207</v>
+        <v>156</v>
       </c>
       <c r="L3" t="n">
-        <v>75</v>
+        <v>35</v>
       </c>
       <c r="M3" t="n">
-        <v>606</v>
+        <v>419</v>
       </c>
       <c r="N3" t="n">
-        <v>4923</v>
+        <v>3724</v>
       </c>
       <c r="O3" t="n">
-        <v>4.28</v>
+        <v>18.32</v>
       </c>
       <c r="P3" t="n">
-        <v>6.34</v>
+        <v>33.42</v>
       </c>
       <c r="Q3" t="n">
-        <v>6.36</v>
+        <v>33.58</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
           <t>Automobiles</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S3" t="n">
+        <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>30.423</v>
+        <v>33.706</v>
       </c>
       <c r="U3" t="n">
         <v>2</v>
       </c>
       <c r="V3" s="1" t="n">
-        <v>85.70999999999999</v>
+        <v>83.33</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>HEROMOTOCO</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -723,150 +726,146 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>24.97</v>
+        <v>10.31</v>
       </c>
       <c r="D4" t="n">
-        <v>26.17</v>
+        <v>86.13</v>
       </c>
       <c r="E4" t="n">
-        <v>22.17</v>
+        <v>21.14</v>
       </c>
       <c r="F4" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="G4" t="n">
-        <v>117</v>
+        <v>37.19</v>
       </c>
       <c r="H4" t="n">
-        <v>0.72</v>
+        <v>1.44</v>
       </c>
       <c r="I4" t="n">
-        <v>6558</v>
+        <v>6751</v>
       </c>
       <c r="J4" t="n">
-        <v>2834</v>
+        <v>1828</v>
       </c>
       <c r="K4" t="n">
-        <v>156</v>
+        <v>207</v>
       </c>
       <c r="L4" t="n">
-        <v>35</v>
+        <v>75</v>
       </c>
       <c r="M4" t="n">
-        <v>419</v>
+        <v>606</v>
       </c>
       <c r="N4" t="n">
-        <v>3724</v>
+        <v>4923</v>
       </c>
       <c r="O4" t="n">
-        <v>8.539999999999999</v>
+        <v>6.68</v>
       </c>
       <c r="P4" t="n">
-        <v>20.08</v>
+        <v>8.92</v>
       </c>
       <c r="Q4" t="n">
-        <v>23.83</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
           <t>Automobiles</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S4" t="n">
+        <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>29.082</v>
+        <v>31.419</v>
       </c>
       <c r="U4" t="n">
         <v>3</v>
       </c>
       <c r="V4" s="2" t="n">
-        <v>71.43000000000001</v>
+        <v>66.67</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>MARUTI</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>TTM</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="3" t="n">
         <v>9.66</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="3" t="n">
         <v>13.61</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="3" t="n">
         <v>15.75</v>
       </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
+      <c r="F5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
         <v>116.83</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="3" t="n">
         <v>1.23</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" s="3" t="n">
         <v>28666</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J5" s="3" t="n">
         <v>11865</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" s="3" t="n">
         <v>446</v>
       </c>
-      <c r="L5" t="n">
+      <c r="L5" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="M5" t="n">
+      <c r="M5" s="3" t="n">
         <v>119</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N5" s="3" t="n">
         <v>16801</v>
       </c>
-      <c r="O5" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="P5" t="n">
-        <v>15.57</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>15.16</v>
-      </c>
-      <c r="R5" t="inlineStr">
+      <c r="O5" s="3" t="n">
+        <v>19.85</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>33.69</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>32.43</v>
+      </c>
+      <c r="R5" s="3" t="inlineStr">
         <is>
           <t>Automobiles</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T5" t="n">
-        <v>24.336</v>
-      </c>
-      <c r="U5" t="n">
+      <c r="S5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="T5" s="3" t="n">
+        <v>29.85</v>
+      </c>
+      <c r="U5" s="3" t="n">
         <v>4</v>
       </c>
       <c r="V5" s="2" t="n">
-        <v>57.14</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TVSMOTOR</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -875,74 +874,72 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>4.88</v>
+        <v>8.92</v>
       </c>
       <c r="D6" t="n">
-        <v>14.43</v>
+        <v>18.65</v>
       </c>
       <c r="E6" t="n">
-        <v>26.22</v>
+        <v>18.54</v>
       </c>
       <c r="F6" t="n">
-        <v>3.83</v>
+        <v>1.64</v>
       </c>
       <c r="G6" t="n">
-        <v>3.05</v>
+        <v>3.7</v>
       </c>
       <c r="H6" t="n">
-        <v>0.93</v>
+        <v>0.59</v>
       </c>
       <c r="I6" t="n">
-        <v>-252</v>
+        <v>-15</v>
       </c>
       <c r="J6" t="n">
-        <v>1001</v>
+        <v>5615</v>
       </c>
       <c r="K6" t="n">
-        <v>42</v>
+        <v>95</v>
       </c>
       <c r="L6" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="M6" t="n">
-        <v>26006</v>
+        <v>108647</v>
       </c>
       <c r="N6" t="n">
-        <v>-1253</v>
+        <v>-5630</v>
       </c>
       <c r="O6" t="n">
-        <v>15.63</v>
+        <v>18.38</v>
       </c>
       <c r="P6" t="n">
-        <v>21.72</v>
+        <v>71.27</v>
       </c>
       <c r="Q6" t="n">
-        <v>21.65</v>
+        <v>58.64</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
           <t>Automobiles</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S6" t="n">
+        <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>18.437</v>
+        <v>27.448</v>
       </c>
       <c r="U6" t="n">
         <v>5</v>
       </c>
       <c r="V6" s="2" t="n">
-        <v>42.86</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TATAMOTORS</t>
+          <t>TVSMOTOR</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -951,74 +948,72 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>7.68</v>
+        <v>4.88</v>
       </c>
       <c r="D7" t="n">
-        <v>13.75</v>
+        <v>14.43</v>
       </c>
       <c r="E7" t="n">
-        <v>37.46</v>
+        <v>26.22</v>
       </c>
       <c r="F7" t="n">
-        <v>1.26</v>
+        <v>3.83</v>
       </c>
       <c r="G7" t="n">
-        <v>7.59</v>
+        <v>3.05</v>
       </c>
       <c r="H7" t="n">
-        <v>1.19</v>
+        <v>0.93</v>
       </c>
       <c r="I7" t="n">
-        <v>90697</v>
+        <v>-252</v>
       </c>
       <c r="J7" t="n">
-        <v>22782</v>
+        <v>1001</v>
       </c>
       <c r="K7" t="n">
-        <v>99</v>
+        <v>42</v>
       </c>
       <c r="L7" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="M7" t="n">
-        <v>107262</v>
+        <v>26006</v>
       </c>
       <c r="N7" t="n">
-        <v>67915</v>
+        <v>-1253</v>
       </c>
       <c r="O7" t="n">
-        <v>7.31</v>
+        <v>21.9</v>
       </c>
       <c r="P7" t="n">
-        <v>10.71</v>
+        <v>36.23</v>
       </c>
       <c r="Q7" t="n">
-        <v>9.050000000000001</v>
+        <v>34.07</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
           <t>Automobiles</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S7" t="n">
+        <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>18.215</v>
+        <v>22.593</v>
       </c>
       <c r="U7" t="n">
         <v>6</v>
       </c>
-      <c r="V7" s="2" t="n">
-        <v>28.57</v>
+      <c r="V7" s="4" t="n">
+        <v>16.67</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>TATAMOTORS</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1027,69 +1022,57 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>8.92</v>
+        <v>7.68</v>
       </c>
       <c r="D8" t="n">
-        <v>18.65</v>
+        <v>13.75</v>
       </c>
       <c r="E8" t="n">
-        <v>18.54</v>
+        <v>37.46</v>
       </c>
       <c r="F8" t="n">
-        <v>1.64</v>
+        <v>1.26</v>
       </c>
       <c r="G8" t="n">
-        <v>3.7</v>
+        <v>7.59</v>
       </c>
       <c r="H8" t="n">
-        <v>0.59</v>
+        <v>1.19</v>
       </c>
       <c r="I8" t="n">
-        <v>-15</v>
+        <v>90697</v>
       </c>
       <c r="J8" t="n">
-        <v>5615</v>
+        <v>22782</v>
       </c>
       <c r="K8" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="L8" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="M8" t="n">
-        <v>108647</v>
+        <v>107262</v>
       </c>
       <c r="N8" t="n">
-        <v>-5630</v>
+        <v>67915</v>
       </c>
       <c r="O8" t="n">
-        <v>6.48</v>
-      </c>
-      <c r="P8" t="n">
-        <v>10.04</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>9.210000000000001</v>
-      </c>
+        <v>15.21</v>
+      </c>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
           <t>Automobiles</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T8" t="n">
-        <v>12.822</v>
-      </c>
-      <c r="U8" t="n">
-        <v>7</v>
-      </c>
-      <c r="V8" s="3" t="n">
-        <v>14.29</v>
-      </c>
+      <c r="S8" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1135,24 +1118,26 @@
         <v>4923</v>
       </c>
       <c r="O9" t="n">
-        <v>7.72</v>
+        <v>18.32</v>
       </c>
       <c r="P9" t="n">
-        <v>10.71</v>
+        <v>33.555</v>
       </c>
       <c r="Q9" t="n">
-        <v>9.210000000000001</v>
+        <v>33.005</v>
       </c>
       <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
+      <c r="S9" t="n">
+        <v>0</v>
+      </c>
       <c r="T9" t="n">
-        <v>24.336</v>
+        <v>30.6345</v>
       </c>
       <c r="U9" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="V9" s="2" t="n">
-        <v>57.14</v>
+        <v>58.335</v>
       </c>
     </row>
   </sheetData>
@@ -1284,7 +1269,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CANBK</t>
+          <t>BANKBARODA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1293,62 +1278,60 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>13.88</v>
+        <v>16.23</v>
       </c>
       <c r="D2" t="n">
-        <v>40.23</v>
+        <v>37.42</v>
       </c>
       <c r="E2" t="n">
-        <v>16.72</v>
+        <v>15.76</v>
       </c>
       <c r="F2" t="n">
-        <v>14.87</v>
+        <v>12.14</v>
       </c>
       <c r="G2" t="n">
-        <v>1.58</v>
+        <v>1.95</v>
       </c>
       <c r="H2" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="I2" t="n">
-        <v>16796</v>
+        <v>-4989</v>
       </c>
       <c r="J2" t="n">
-        <v>1750</v>
+        <v>1285</v>
       </c>
       <c r="K2" t="n">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="L2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M2" t="n">
-        <v>1369780</v>
+        <v>1453761</v>
       </c>
       <c r="N2" t="n">
-        <v>15046</v>
+        <v>-6274</v>
       </c>
       <c r="O2" t="n">
-        <v>11.02</v>
+        <v>13.69</v>
       </c>
       <c r="P2" t="n">
-        <v>15.32</v>
+        <v>87.78</v>
       </c>
       <c r="Q2" t="n">
-        <v>3.44</v>
+        <v>89.88</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
           <t>Public Sector Banks</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S2" t="n">
+        <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>18.795</v>
+        <v>32.71</v>
       </c>
       <c r="U2" t="n">
         <v>1</v>
@@ -1360,7 +1343,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BANKBARODA</t>
+          <t>CANBK</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1369,62 +1352,60 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>16.23</v>
+        <v>13.88</v>
       </c>
       <c r="D3" t="n">
-        <v>37.42</v>
+        <v>40.23</v>
       </c>
       <c r="E3" t="n">
-        <v>15.76</v>
+        <v>16.72</v>
       </c>
       <c r="F3" t="n">
-        <v>12.14</v>
+        <v>14.87</v>
       </c>
       <c r="G3" t="n">
-        <v>1.95</v>
+        <v>1.58</v>
       </c>
       <c r="H3" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>-4989</v>
+        <v>16796</v>
       </c>
       <c r="J3" t="n">
-        <v>1285</v>
+        <v>1750</v>
       </c>
       <c r="K3" t="n">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="L3" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="M3" t="n">
-        <v>1453761</v>
+        <v>1369780</v>
       </c>
       <c r="N3" t="n">
-        <v>-6274</v>
+        <v>15046</v>
       </c>
       <c r="O3" t="n">
-        <v>10.75</v>
+        <v>14.18</v>
       </c>
       <c r="P3" t="n">
-        <v>12.64</v>
+        <v>53.86</v>
       </c>
       <c r="Q3" t="n">
-        <v>4.5</v>
+        <v>45.65</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
           <t>Public Sector Banks</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S3" t="n">
+        <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>17.094</v>
+        <v>27.135</v>
       </c>
       <c r="U3" t="n">
         <v>2</v>
@@ -1477,89 +1458,85 @@
         <v>-27939</v>
       </c>
       <c r="O4" t="n">
-        <v>8.619999999999999</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="P4" t="n">
-        <v>9.26</v>
+        <v>52.39</v>
       </c>
       <c r="Q4" t="n">
-        <v>-6.19</v>
+        <v>59.67</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
           <t>Public Sector Banks</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S4" t="n">
+        <v>0</v>
       </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>SBIN</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>TTM</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="3" t="n">
         <v>15.86</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="3" t="n">
         <v>-12.6</v>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="n">
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="n">
         <v>0.34</v>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="n">
+      <c r="H5" s="3" t="inlineStr"/>
+      <c r="I5" s="3" t="n">
         <v>25108</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J5" s="3" t="n">
         <v>3476</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="L5" t="n">
+      <c r="L5" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="n">
+      <c r="M5" s="3" t="inlineStr"/>
+      <c r="N5" s="3" t="n">
         <v>21632</v>
       </c>
-      <c r="O5" t="n">
-        <v>8.949999999999999</v>
-      </c>
-      <c r="P5" t="n">
-        <v>12.28</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>9.82</v>
-      </c>
-      <c r="R5" t="inlineStr">
+      <c r="O5" s="3" t="n">
+        <v>13.99</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>32.87</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>33.75</v>
+      </c>
+      <c r="R5" s="3" t="inlineStr">
         <is>
           <t>Public Sector Banks</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
+      <c r="S5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="T5" s="3" t="inlineStr"/>
+      <c r="U5" s="3" t="inlineStr"/>
+      <c r="V5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1605,18 +1582,20 @@
         <v>4386</v>
       </c>
       <c r="O6" t="n">
-        <v>9.85</v>
+        <v>13.84</v>
       </c>
       <c r="P6" t="n">
-        <v>12.46</v>
+        <v>53.125</v>
       </c>
       <c r="Q6" t="n">
-        <v>3.97</v>
+        <v>52.66</v>
       </c>
       <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
       <c r="T6" t="n">
-        <v>17.94450000000001</v>
+        <v>29.9225</v>
       </c>
       <c r="U6" t="n">
         <v>1.5</v>
@@ -1799,26 +1778,24 @@
         <v>24056</v>
       </c>
       <c r="O2" t="n">
-        <v>8.94</v>
+        <v>14.14</v>
       </c>
       <c r="P2" t="n">
-        <v>12.6</v>
+        <v>37.61</v>
       </c>
       <c r="Q2" t="n">
-        <v>11</v>
+        <v>36.78</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
           <t>Steel</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S2" t="n">
+        <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>37.616</v>
+        <v>43.658</v>
       </c>
       <c r="U2" t="n">
         <v>1</v>
@@ -1830,7 +1807,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>JINDALSTEL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1839,74 +1816,72 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.95</v>
+        <v>10.12</v>
       </c>
       <c r="D3" t="n">
-        <v>13.2</v>
+        <v>20.65</v>
       </c>
       <c r="E3" t="n">
-        <v>11.55</v>
+        <v>13.41</v>
       </c>
       <c r="F3" t="n">
-        <v>1.13</v>
+        <v>0.37</v>
       </c>
       <c r="G3" t="n">
-        <v>2.71</v>
+        <v>8.09</v>
       </c>
       <c r="H3" t="n">
-        <v>0.77</v>
+        <v>0.64</v>
       </c>
       <c r="I3" t="n">
-        <v>26545</v>
+        <v>14352</v>
       </c>
       <c r="J3" t="n">
-        <v>14467</v>
+        <v>8344</v>
       </c>
       <c r="K3" t="n">
-        <v>14</v>
+        <v>50</v>
       </c>
       <c r="L3" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="M3" t="n">
-        <v>87984</v>
+        <v>16472</v>
       </c>
       <c r="N3" t="n">
-        <v>12078</v>
+        <v>6008</v>
       </c>
       <c r="O3" t="n">
-        <v>13.26</v>
+        <v>9.67</v>
       </c>
       <c r="P3" t="n">
-        <v>11.17</v>
+        <v>4.35</v>
       </c>
       <c r="Q3" t="n">
-        <v>11</v>
+        <v>8.56</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
           <t>Steel</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S3" t="n">
+        <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>11.935</v>
+        <v>11.679</v>
       </c>
       <c r="U3" t="n">
         <v>2</v>
       </c>
-      <c r="V3" s="2" t="n">
-        <v>66.67</v>
+      <c r="V3" s="1" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>JINDALSTEL</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1915,135 +1890,141 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>10.12</v>
+        <v>1.95</v>
       </c>
       <c r="D4" t="n">
-        <v>20.65</v>
+        <v>13.2</v>
       </c>
       <c r="E4" t="n">
-        <v>13.41</v>
+        <v>11.55</v>
       </c>
       <c r="F4" t="n">
-        <v>0.37</v>
+        <v>1.13</v>
       </c>
       <c r="G4" t="n">
-        <v>8.09</v>
+        <v>2.71</v>
       </c>
       <c r="H4" t="n">
-        <v>0.64</v>
+        <v>0.77</v>
       </c>
       <c r="I4" t="n">
-        <v>14352</v>
+        <v>26545</v>
       </c>
       <c r="J4" t="n">
-        <v>8344</v>
+        <v>14467</v>
       </c>
       <c r="K4" t="n">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="L4" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="M4" t="n">
-        <v>16472</v>
+        <v>87984</v>
       </c>
       <c r="N4" t="n">
-        <v>6008</v>
+        <v>12078</v>
       </c>
       <c r="O4" t="n">
-        <v>8.029999999999999</v>
+        <v>20.85</v>
       </c>
       <c r="P4" t="n">
-        <v>4.59</v>
+        <v>-19.46</v>
       </c>
       <c r="Q4" t="n">
-        <v>4.06</v>
+        <v>-19.29</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
           <t>Steel</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S4" t="n">
+        <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>11.399</v>
+        <v>7.327000000000001</v>
       </c>
       <c r="U4" t="n">
         <v>3</v>
       </c>
       <c r="V4" s="2" t="n">
-        <v>33.33</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>TATASTEEL</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>TTM</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="3" t="n">
         <v>1.14</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="3" t="n">
         <v>11.45</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="3" t="n">
         <v>-5.33</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="3" t="n">
         <v>0.95</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="3" t="n">
         <v>3.47</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="3" t="n">
         <v>0.85</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" s="3" t="n">
         <v>34554</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J5" s="3" t="n">
         <v>14253</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="L5" t="n">
+      <c r="L5" s="3" t="n">
         <v>-101</v>
       </c>
-      <c r="M5" t="n">
+      <c r="M5" s="3" t="n">
         <v>87082</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N5" s="3" t="n">
         <v>20301</v>
       </c>
-      <c r="O5" t="n">
-        <v>4.21</v>
-      </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr">
+      <c r="O5" s="3" t="n">
+        <v>9.050000000000001</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>-25.47</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>-24.02</v>
+      </c>
+      <c r="R5" s="3" t="inlineStr">
         <is>
           <t>Steel</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
+      <c r="S5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="T5" s="3" t="n">
+        <v>-2.725</v>
+      </c>
+      <c r="U5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="V5" s="2" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2089,24 +2070,26 @@
         <v>16189.5</v>
       </c>
       <c r="O6" t="n">
-        <v>8.484999999999999</v>
+        <v>11.905</v>
       </c>
       <c r="P6" t="n">
-        <v>11.17</v>
+        <v>-7.555000000000001</v>
       </c>
       <c r="Q6" t="n">
-        <v>11</v>
+        <v>-5.364999999999999</v>
       </c>
       <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
       <c r="T6" t="n">
-        <v>11.935</v>
+        <v>9.503</v>
       </c>
       <c r="U6" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="V6" s="2" t="n">
-        <v>66.67</v>
+        <v>62.5</v>
       </c>
     </row>
   </sheetData>
@@ -2236,75 +2219,73 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>BAJFINANCE</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>TTM</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="3" t="n">
         <v>24.71</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="3" t="n">
         <v>30.42</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="3" t="n">
         <v>18.84</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="3" t="n">
         <v>3.82</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="3" t="n">
         <v>654.38</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="3" t="n">
         <v>0.15</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="3" t="n">
         <v>-65589</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" s="3" t="n">
         <v>7171</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" s="3" t="n">
         <v>248</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L2" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M2" s="3" t="n">
         <v>293346</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N2" s="3" t="n">
         <v>-72760</v>
       </c>
-      <c r="O2" t="n">
-        <v>27.72</v>
-      </c>
-      <c r="P2" t="n">
-        <v>32.86</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>29.99</v>
-      </c>
-      <c r="R2" t="inlineStr">
+      <c r="O2" s="3" t="n">
+        <v>23.61</v>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="Q2" s="3" t="n">
+        <v>35.76</v>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t>Consumer Finance</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T2" t="n">
-        <v>292.543</v>
-      </c>
-      <c r="U2" t="n">
+      <c r="S2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2" s="3" t="n">
+        <v>292.4690000000001</v>
+      </c>
+      <c r="U2" s="3" t="n">
         <v>1</v>
       </c>
       <c r="V2" s="1" t="n">
@@ -2359,26 +2340,24 @@
         <v>-35683</v>
       </c>
       <c r="O3" t="n">
-        <v>19.82</v>
+        <v>23.79</v>
       </c>
       <c r="P3" t="n">
-        <v>23.43</v>
+        <v>26.15</v>
       </c>
       <c r="Q3" t="n">
-        <v>22.57</v>
+        <v>24.74</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
           <t>Consumer Finance</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S3" t="n">
+        <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>21.629</v>
+        <v>22.967</v>
       </c>
       <c r="U3" t="n">
         <v>2</v>
@@ -2435,26 +2414,24 @@
         <v>-31101</v>
       </c>
       <c r="O4" t="n">
-        <v>15.59</v>
+        <v>22.99</v>
       </c>
       <c r="P4" t="n">
-        <v>16.82</v>
+        <v>39.46</v>
       </c>
       <c r="Q4" t="n">
-        <v>12.63</v>
+        <v>29.1</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
           <t>Consumer Finance</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S4" t="n">
+        <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>16.87</v>
+        <v>22.878</v>
       </c>
       <c r="U4" t="n">
         <v>3</v>
@@ -2507,18 +2484,20 @@
         <v>-35683</v>
       </c>
       <c r="O5" t="n">
-        <v>19.82</v>
+        <v>23.61</v>
       </c>
       <c r="P5" t="n">
-        <v>23.43</v>
+        <v>36.6</v>
       </c>
       <c r="Q5" t="n">
-        <v>22.57</v>
+        <v>29.1</v>
       </c>
       <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
+      <c r="S5" t="n">
+        <v>0</v>
+      </c>
       <c r="T5" t="n">
-        <v>21.629</v>
+        <v>22.967</v>
       </c>
       <c r="U5" t="n">
         <v>2</v>
@@ -2701,26 +2680,24 @@
         <v>17179</v>
       </c>
       <c r="O2" t="n">
-        <v>7.48</v>
+        <v>11.13</v>
       </c>
       <c r="P2" t="n">
-        <v>8.640000000000001</v>
+        <v>11.69</v>
       </c>
       <c r="Q2" t="n">
-        <v>8.52</v>
+        <v>9.82</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
           <t>FMCG</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S2" t="n">
+        <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>55.279</v>
+        <v>56.619</v>
       </c>
       <c r="U2" t="n">
         <v>1</v>
@@ -2777,26 +2754,24 @@
         <v>4175</v>
       </c>
       <c r="O3" t="n">
-        <v>6.69</v>
+        <v>7.64</v>
       </c>
       <c r="P3" t="n">
-        <v>9.51</v>
+        <v>11.92</v>
       </c>
       <c r="Q3" t="n">
-        <v>9.07</v>
+        <v>11.5</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
           <t>FMCG</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S3" t="n">
+        <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>47.45</v>
+        <v>48.12199999999999</v>
       </c>
       <c r="U3" t="n">
         <v>2</v>
@@ -2806,75 +2781,73 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>HINDUNILVR</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>TTM</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="3" t="n">
         <v>17.17</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="3" t="n">
         <v>76.45</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="3" t="n">
         <v>20.07</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="3" t="n">
         <v>0.03</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="3" t="n">
         <v>32.8</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="3" t="n">
         <v>0.79</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="3" t="n">
         <v>20793</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J4" s="3" t="n">
         <v>5324</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" s="3" t="n">
         <v>46</v>
       </c>
-      <c r="L4" t="n">
+      <c r="L4" s="3" t="n">
         <v>96</v>
       </c>
-      <c r="M4" t="n">
+      <c r="M4" s="3" t="n">
         <v>1484</v>
       </c>
-      <c r="N4" t="n">
+      <c r="N4" s="3" t="n">
         <v>15469</v>
       </c>
-      <c r="O4" t="n">
-        <v>7.27</v>
-      </c>
-      <c r="P4" t="n">
-        <v>8.970000000000001</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>8.130000000000001</v>
-      </c>
-      <c r="R4" t="inlineStr">
+      <c r="O4" s="3" t="n">
+        <v>7.44</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="Q4" s="3" t="n">
+        <v>7.85</v>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>FMCG</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T4" t="n">
-        <v>30.318</v>
-      </c>
-      <c r="U4" t="n">
+      <c r="S4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="T4" s="3" t="n">
+        <v>30.096</v>
+      </c>
+      <c r="U4" s="3" t="n">
         <v>3</v>
       </c>
       <c r="V4" s="2" t="n">
@@ -2929,26 +2902,24 @@
         <v>2573</v>
       </c>
       <c r="O5" t="n">
-        <v>8.92</v>
+        <v>7.04</v>
       </c>
       <c r="P5" t="n">
-        <v>19.15</v>
+        <v>3.56</v>
       </c>
       <c r="Q5" t="n">
-        <v>19.03</v>
+        <v>3.69</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
           <t>FMCG</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S5" t="n">
+        <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>27.69699999999999</v>
+        <v>24.203</v>
       </c>
       <c r="U5" t="n">
         <v>4</v>
@@ -3005,26 +2976,24 @@
         <v>2013</v>
       </c>
       <c r="O6" t="n">
-        <v>6.07</v>
+        <v>6.81</v>
       </c>
       <c r="P6" t="n">
-        <v>7.18</v>
+        <v>0.95</v>
       </c>
       <c r="Q6" t="n">
-        <v>7.93</v>
+        <v>0</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
           <t>FMCG</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S6" t="n">
+        <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>14.352</v>
+        <v>13.254</v>
       </c>
       <c r="U6" t="n">
         <v>5</v>
@@ -3081,31 +3050,29 @@
         <v>1937</v>
       </c>
       <c r="O7" t="n">
-        <v>6.86</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="P7" t="n">
-        <v>8.390000000000001</v>
+        <v>5.91</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.95</v>
+        <v>7.46</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
           <t>FMCG</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S7" t="n">
+        <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>10.857</v>
+        <v>10.763</v>
       </c>
       <c r="U7" t="n">
         <v>6</v>
       </c>
-      <c r="V7" s="3" t="n">
+      <c r="V7" s="4" t="n">
         <v>16.67</v>
       </c>
     </row>
@@ -3157,7 +3124,7 @@
         <v>2070</v>
       </c>
       <c r="O8" t="n">
-        <v>6.82</v>
+        <v>6.43</v>
       </c>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
@@ -3166,10 +3133,8 @@
           <t>FMCG</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S8" t="n">
+        <v>0</v>
       </c>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
@@ -3219,18 +3184,20 @@
         <v>2573</v>
       </c>
       <c r="O9" t="n">
-        <v>6.86</v>
+        <v>7.44</v>
       </c>
       <c r="P9" t="n">
-        <v>8.805</v>
+        <v>6.800000000000001</v>
       </c>
       <c r="Q9" t="n">
-        <v>8.324999999999999</v>
+        <v>7.654999999999999</v>
       </c>
       <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
+      <c r="S9" t="n">
+        <v>0</v>
+      </c>
       <c r="T9" t="n">
-        <v>29.0075</v>
+        <v>27.1495</v>
       </c>
       <c r="U9" t="n">
         <v>3.5</v>
@@ -3366,75 +3333,73 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>TCS</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>TTM</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="3" t="n">
         <v>19.44</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="3" t="n">
         <v>26.81</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="3" t="n">
         <v>50.94</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="3" t="n">
         <v>0.09</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="3" t="n">
         <v>90.17</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="3" t="n">
         <v>1.66</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="3" t="n">
         <v>50429</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" s="3" t="n">
         <v>6091</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" s="3" t="n">
         <v>135</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L2" s="3" t="n">
         <v>58</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M2" s="3" t="n">
         <v>8021</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N2" s="3" t="n">
         <v>44338</v>
       </c>
-      <c r="O2" t="n">
-        <v>12.25</v>
-      </c>
-      <c r="P2" t="n">
-        <v>10.96</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>11.64</v>
-      </c>
-      <c r="R2" t="inlineStr">
+      <c r="O2" s="3" t="n">
+        <v>11.32</v>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>10.76</v>
+      </c>
+      <c r="Q2" s="3" t="n">
+        <v>11.29</v>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t>IT Services</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T2" t="n">
-        <v>33.97199999999999</v>
-      </c>
-      <c r="U2" t="n">
+      <c r="S2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2" s="3" t="n">
+        <v>33.746</v>
+      </c>
+      <c r="U2" s="3" t="n">
         <v>1</v>
       </c>
       <c r="V2" s="1" t="n">
@@ -3444,7 +3409,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3453,62 +3418,60 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>17.31</v>
+        <v>14.82</v>
       </c>
       <c r="D3" t="n">
-        <v>23.84</v>
+        <v>21.8</v>
       </c>
       <c r="E3" t="n">
-        <v>29.79</v>
+        <v>23.01</v>
       </c>
       <c r="F3" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="G3" t="n">
-        <v>102.08</v>
+        <v>41.87</v>
       </c>
       <c r="H3" t="n">
-        <v>1.13</v>
+        <v>1.11</v>
       </c>
       <c r="I3" t="n">
-        <v>30303</v>
+        <v>29056</v>
       </c>
       <c r="J3" t="n">
-        <v>5093</v>
+        <v>6608</v>
       </c>
       <c r="K3" t="n">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="L3" t="n">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="M3" t="n">
-        <v>8359</v>
+        <v>5758</v>
       </c>
       <c r="N3" t="n">
-        <v>25210</v>
+        <v>22448</v>
       </c>
       <c r="O3" t="n">
-        <v>12.16</v>
+        <v>38.72</v>
       </c>
       <c r="P3" t="n">
-        <v>9.390000000000001</v>
+        <v>32.15</v>
       </c>
       <c r="Q3" t="n">
-        <v>10.15</v>
+        <v>33.22</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
           <t>IT Services</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S3" t="n">
+        <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>26.739</v>
+        <v>30.127</v>
       </c>
       <c r="U3" t="n">
         <v>2</v>
@@ -3520,7 +3483,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LTIM</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3529,62 +3492,60 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>12.32</v>
+        <v>17.31</v>
       </c>
       <c r="D4" t="n">
-        <v>17.33</v>
+        <v>23.84</v>
       </c>
       <c r="E4" t="n">
-        <v>22.9</v>
+        <v>29.79</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="G4" t="n">
-        <v>26.36</v>
+        <v>102.08</v>
       </c>
       <c r="H4" t="n">
-        <v>1.29</v>
+        <v>1.13</v>
       </c>
       <c r="I4" t="n">
-        <v>9588</v>
+        <v>30303</v>
       </c>
       <c r="J4" t="n">
-        <v>3918</v>
+        <v>5093</v>
       </c>
       <c r="K4" t="n">
-        <v>154</v>
+        <v>67</v>
       </c>
       <c r="L4" t="n">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="M4" t="n">
-        <v>2071</v>
+        <v>8359</v>
       </c>
       <c r="N4" t="n">
-        <v>5670</v>
+        <v>25210</v>
       </c>
       <c r="O4" t="n">
-        <v>20.78</v>
+        <v>12.33</v>
       </c>
       <c r="P4" t="n">
-        <v>19.09</v>
+        <v>9.27</v>
       </c>
       <c r="Q4" t="n">
-        <v>-1.01</v>
+        <v>10.46</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
           <t>IT Services</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S4" t="n">
+        <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>21.633</v>
+        <v>26.749</v>
       </c>
       <c r="U4" t="n">
         <v>3</v>
@@ -3596,7 +3557,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>LTIM</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3605,62 +3566,60 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>14.82</v>
+        <v>12.32</v>
       </c>
       <c r="D5" t="n">
-        <v>21.8</v>
+        <v>17.33</v>
       </c>
       <c r="E5" t="n">
-        <v>23.01</v>
+        <v>22.9</v>
       </c>
       <c r="F5" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="G5" t="n">
-        <v>41.87</v>
+        <v>26.36</v>
       </c>
       <c r="H5" t="n">
-        <v>1.11</v>
+        <v>1.29</v>
       </c>
       <c r="I5" t="n">
-        <v>29056</v>
+        <v>9588</v>
       </c>
       <c r="J5" t="n">
-        <v>6608</v>
+        <v>3918</v>
       </c>
       <c r="K5" t="n">
-        <v>63</v>
+        <v>154</v>
       </c>
       <c r="L5" t="n">
-        <v>90</v>
+        <v>42</v>
       </c>
       <c r="M5" t="n">
-        <v>5758</v>
+        <v>2071</v>
       </c>
       <c r="N5" t="n">
-        <v>22448</v>
+        <v>5670</v>
       </c>
       <c r="O5" t="n">
-        <v>7.66</v>
+        <v>31.62</v>
       </c>
       <c r="P5" t="n">
-        <v>5.88</v>
+        <v>23.95</v>
       </c>
       <c r="Q5" t="n">
-        <v>6.38</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
           <t>IT Services</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S5" t="n">
+        <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>18.661</v>
+        <v>24.773</v>
       </c>
       <c r="U5" t="n">
         <v>4</v>
@@ -3717,31 +3676,29 @@
         <v>6376</v>
       </c>
       <c r="O6" t="n">
-        <v>18.46</v>
+        <v>8.51</v>
       </c>
       <c r="P6" t="n">
-        <v>9.24</v>
+        <v>-3.5</v>
       </c>
       <c r="Q6" t="n">
-        <v>3.55</v>
+        <v>-4.66</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
           <t>IT Services</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S6" t="n">
+        <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>11.357</v>
+        <v>6.819</v>
       </c>
       <c r="U6" t="n">
         <v>5</v>
       </c>
-      <c r="V6" s="3" t="n">
+      <c r="V6" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3789,18 +3746,20 @@
         <v>22448</v>
       </c>
       <c r="O7" t="n">
-        <v>12.25</v>
+        <v>12.33</v>
       </c>
       <c r="P7" t="n">
-        <v>9.390000000000001</v>
+        <v>10.76</v>
       </c>
       <c r="Q7" t="n">
-        <v>6.38</v>
+        <v>10.46</v>
       </c>
       <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
       <c r="T7" t="n">
-        <v>21.633</v>
+        <v>26.749</v>
       </c>
       <c r="U7" t="n">
         <v>3</v>
@@ -3936,73 +3895,71 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>LICI</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>TTM</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="3" t="n">
         <v>4.63</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="3" t="n">
         <v>2.88</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="3" t="n">
         <v>49.45</v>
       </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
+      <c r="F2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="3" t="n">
         <v>371.94</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="3" t="n">
         <v>0.16</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="3" t="n">
         <v>51391</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" s="3" t="n">
         <v>25269</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" s="3" t="n">
         <v>66</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L2" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="n">
+      <c r="M2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="3" t="n">
         <v>26122</v>
       </c>
-      <c r="O2" t="n">
-        <v>7.78</v>
-      </c>
-      <c r="P2" t="n">
-        <v>58.38</v>
-      </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr">
+      <c r="O2" s="3" t="n">
+        <v>6.72</v>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>93.23999999999999</v>
+      </c>
+      <c r="Q2" s="3" t="inlineStr"/>
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t>Life Insurance</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="T2" t="n">
-        <v>66.03500000000001</v>
-      </c>
-      <c r="U2" t="n">
+      <c r="S2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2" s="3" t="n">
+        <v>72.795</v>
+      </c>
+      <c r="U2" s="3" t="n">
         <v>1</v>
       </c>
       <c r="V2" s="1" t="n">
@@ -4057,26 +4014,24 @@
         <v>10721</v>
       </c>
       <c r="O3" t="n">
-        <v>17.84</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="P3" t="n">
-        <v>12.03</v>
+        <v>6.44</v>
       </c>
       <c r="Q3" t="n">
-        <v>12.25</v>
+        <v>3.39</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
           <t>Life Insurance</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S3" t="n">
+        <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>48.318</v>
+        <v>45.422</v>
       </c>
       <c r="U3" t="n">
         <v>2</v>
@@ -4133,26 +4088,24 @@
         <v>29122</v>
       </c>
       <c r="O4" t="n">
-        <v>19.81</v>
+        <v>12.26</v>
       </c>
       <c r="P4" t="n">
-        <v>11.83</v>
+        <v>13.44</v>
       </c>
       <c r="Q4" t="n">
-        <v>12.25</v>
+        <v>12.47</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
           <t>Life Insurance</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S4" t="n">
+        <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>34.209</v>
+        <v>33.021</v>
       </c>
       <c r="U4" t="n">
         <v>3</v>
@@ -4209,26 +4162,24 @@
         <v>-7315</v>
       </c>
       <c r="O5" t="n">
-        <v>11.95</v>
+        <v>-1.73</v>
       </c>
       <c r="P5" t="n">
-        <v>-3.61</v>
+        <v>0.47</v>
       </c>
       <c r="Q5" t="n">
-        <v>-3.7</v>
+        <v>0</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
           <t>Life Insurance</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S5" t="n">
+        <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>27.495</v>
+        <v>25.575</v>
       </c>
       <c r="U5" t="n">
         <v>4</v>
@@ -4281,18 +4232,20 @@
         <v>18421.5</v>
       </c>
       <c r="O6" t="n">
-        <v>14.895</v>
+        <v>7.834999999999999</v>
       </c>
       <c r="P6" t="n">
-        <v>11.93</v>
+        <v>9.94</v>
       </c>
       <c r="Q6" t="n">
-        <v>12.25</v>
+        <v>3.39</v>
       </c>
       <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
       <c r="T6" t="n">
-        <v>41.2635</v>
+        <v>39.2215</v>
       </c>
       <c r="U6" t="n">
         <v>2.5</v>
@@ -4430,7 +4383,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4439,62 +4392,60 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3.08</v>
+        <v>6.42</v>
       </c>
       <c r="D2" t="n">
-        <v>5.96</v>
+        <v>13.04</v>
       </c>
       <c r="E2" t="n">
-        <v>35.51</v>
+        <v>16.94</v>
       </c>
       <c r="F2" t="n">
-        <v>0.72</v>
+        <v>0.45</v>
       </c>
       <c r="G2" t="n">
-        <v>8.130000000000001</v>
+        <v>7.97</v>
       </c>
       <c r="H2" t="n">
-        <v>2.21</v>
+        <v>0.83</v>
       </c>
       <c r="I2" t="n">
-        <v>46457</v>
+        <v>156466</v>
       </c>
       <c r="J2" t="n">
-        <v>10521</v>
+        <v>57203</v>
       </c>
       <c r="K2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="L2" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="M2" t="n">
-        <v>54599</v>
+        <v>153181</v>
       </c>
       <c r="N2" t="n">
-        <v>35936</v>
+        <v>99263</v>
       </c>
       <c r="O2" t="n">
-        <v>5.21</v>
+        <v>21.34</v>
       </c>
       <c r="P2" t="n">
-        <v>17.74</v>
+        <v>18.64</v>
       </c>
       <c r="Q2" t="n">
-        <v>18.92</v>
+        <v>26.22</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
           <t>Oil &amp; Gas</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S2" t="n">
+        <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>18.347</v>
+        <v>17.692</v>
       </c>
       <c r="U2" t="n">
         <v>1</v>
@@ -4506,7 +4457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>GAIL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4515,62 +4466,60 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>6.42</v>
+        <v>8.48</v>
       </c>
       <c r="D3" t="n">
-        <v>13.04</v>
+        <v>12.33</v>
       </c>
       <c r="E3" t="n">
-        <v>16.94</v>
+        <v>12.86</v>
       </c>
       <c r="F3" t="n">
-        <v>0.45</v>
+        <v>0.28</v>
       </c>
       <c r="G3" t="n">
-        <v>7.97</v>
+        <v>26.84</v>
       </c>
       <c r="H3" t="n">
-        <v>0.83</v>
+        <v>1.07</v>
       </c>
       <c r="I3" t="n">
-        <v>156466</v>
+        <v>20812</v>
       </c>
       <c r="J3" t="n">
-        <v>57203</v>
+        <v>8226</v>
       </c>
       <c r="K3" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="L3" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="M3" t="n">
-        <v>153181</v>
+        <v>21794</v>
       </c>
       <c r="N3" t="n">
-        <v>99263</v>
+        <v>12586</v>
       </c>
       <c r="O3" t="n">
-        <v>12.4</v>
+        <v>24.1</v>
       </c>
       <c r="P3" t="n">
-        <v>4.84</v>
+        <v>17.08</v>
       </c>
       <c r="Q3" t="n">
-        <v>4.71</v>
+        <v>18.92</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
           <t>Oil &amp; Gas</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S3" t="n">
+        <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>13.144</v>
+        <v>16.604</v>
       </c>
       <c r="U3" t="n">
         <v>2</v>
@@ -4582,7 +4531,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>IOC</t>
+          <t>BPCL</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4591,62 +4540,60 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1.43</v>
+        <v>3.08</v>
       </c>
       <c r="D4" t="n">
-        <v>4.32</v>
+        <v>5.96</v>
       </c>
       <c r="E4" t="n">
-        <v>23.53</v>
+        <v>35.51</v>
       </c>
       <c r="F4" t="n">
         <v>0.72</v>
       </c>
       <c r="G4" t="n">
-        <v>4.36</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>1.61</v>
+        <v>2.21</v>
       </c>
       <c r="I4" t="n">
-        <v>102563</v>
+        <v>46457</v>
       </c>
       <c r="J4" t="n">
-        <v>31464</v>
+        <v>10521</v>
       </c>
       <c r="K4" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="L4" t="n">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="M4" t="n">
-        <v>132628</v>
+        <v>54599</v>
       </c>
       <c r="N4" t="n">
-        <v>71099</v>
+        <v>35936</v>
       </c>
       <c r="O4" t="n">
-        <v>4.26</v>
+        <v>17.96</v>
       </c>
       <c r="P4" t="n">
-        <v>9.609999999999999</v>
+        <v>-5.63</v>
       </c>
       <c r="Q4" t="n">
-        <v>8.52</v>
+        <v>-3.56</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
           <t>Oil &amp; Gas</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S4" t="n">
+        <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>12.809</v>
+        <v>16.223</v>
       </c>
       <c r="U4" t="n">
         <v>3</v>
@@ -4656,75 +4603,73 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>GAIL</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>TTM</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>8.48</v>
-      </c>
-      <c r="D5" t="n">
-        <v>12.33</v>
-      </c>
-      <c r="E5" t="n">
-        <v>12.86</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="G5" t="n">
-        <v>26.84</v>
-      </c>
-      <c r="H5" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="I5" t="n">
-        <v>20812</v>
-      </c>
-      <c r="J5" t="n">
-        <v>8226</v>
-      </c>
-      <c r="K5" t="n">
-        <v>18</v>
-      </c>
-      <c r="L5" t="n">
-        <v>37</v>
-      </c>
-      <c r="M5" t="n">
-        <v>21794</v>
-      </c>
-      <c r="N5" t="n">
-        <v>12586</v>
-      </c>
-      <c r="O5" t="n">
-        <v>8.529999999999999</v>
-      </c>
-      <c r="P5" t="n">
-        <v>8.44</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>9.59</v>
-      </c>
-      <c r="R5" t="inlineStr">
+      <c r="C5" s="3" t="n">
+        <v>8.51</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>17.46</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>9.960000000000001</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>7.61</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>272369</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>113581</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>458991</v>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>158788</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>19.15</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>10.44</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>6.94</v>
+      </c>
+      <c r="R5" s="3" t="inlineStr">
         <is>
           <t>Oil &amp; Gas</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T5" t="n">
-        <v>11.762</v>
-      </c>
-      <c r="U5" t="n">
+      <c r="S5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="T5" s="3" t="n">
+        <v>13.293</v>
+      </c>
+      <c r="U5" s="3" t="n">
         <v>4</v>
       </c>
       <c r="V5" s="2" t="n">
@@ -4734,7 +4679,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>IOC</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4743,67 +4688,65 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>8.51</v>
+        <v>1.43</v>
       </c>
       <c r="D6" t="n">
-        <v>17.46</v>
+        <v>4.32</v>
       </c>
       <c r="E6" t="n">
-        <v>9.960000000000001</v>
+        <v>23.53</v>
       </c>
       <c r="F6" t="n">
-        <v>0.58</v>
+        <v>0.72</v>
       </c>
       <c r="G6" t="n">
-        <v>7.61</v>
+        <v>4.36</v>
       </c>
       <c r="H6" t="n">
-        <v>0.51</v>
+        <v>1.61</v>
       </c>
       <c r="I6" t="n">
-        <v>272369</v>
+        <v>102563</v>
       </c>
       <c r="J6" t="n">
-        <v>113581</v>
+        <v>31464</v>
       </c>
       <c r="K6" t="n">
-        <v>51</v>
+        <v>8</v>
       </c>
       <c r="L6" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="M6" t="n">
-        <v>458991</v>
+        <v>132628</v>
       </c>
       <c r="N6" t="n">
-        <v>158788</v>
+        <v>71099</v>
       </c>
       <c r="O6" t="n">
-        <v>7.47</v>
+        <v>20.27</v>
       </c>
       <c r="P6" t="n">
-        <v>11.83</v>
+        <v>-15.86</v>
       </c>
       <c r="Q6" t="n">
-        <v>10.74</v>
+        <v>-14.54</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
           <t>Oil &amp; Gas</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="S6" t="n">
+        <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>11.235</v>
+        <v>10.917</v>
       </c>
       <c r="U6" t="n">
         <v>5</v>
       </c>
-      <c r="V6" s="3" t="n">
+      <c r="V6" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4851,18 +4794,20 @@
         <v>71099</v>
       </c>
       <c r="O7" t="n">
-        <v>7.47</v>
+        <v>20.27</v>
       </c>
       <c r="P7" t="n">
-        <v>9.609999999999999</v>
+        <v>10.44</v>
       </c>
       <c r="Q7" t="n">
-        <v>9.59</v>
+        <v>6.94</v>
       </c>
       <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
       <c r="T7" t="n">
-        <v>12.809</v>
+        <v>16.223</v>
       </c>
       <c r="U7" t="n">
         <v>3</v>
@@ -5045,26 +4990,24 @@
         <v>1261</v>
       </c>
       <c r="O2" t="n">
-        <v>12.28</v>
+        <v>5.44</v>
       </c>
       <c r="P2" t="n">
-        <v>9.74</v>
+        <v>-1.92</v>
       </c>
       <c r="Q2" t="n">
-        <v>9.59</v>
+        <v>-2.06</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
           <t>Pharmaceuticals</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S2" t="n">
+        <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>77.2</v>
+        <v>73.5</v>
       </c>
       <c r="U2" t="n">
         <v>1</v>
@@ -5121,26 +5064,24 @@
         <v>4134</v>
       </c>
       <c r="O3" t="n">
-        <v>10.35</v>
+        <v>8.93</v>
       </c>
       <c r="P3" t="n">
-        <v>10.26</v>
+        <v>20.2</v>
       </c>
       <c r="Q3" t="n">
-        <v>10.36</v>
+        <v>19.9</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
           <t>Pharmaceuticals</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S3" t="n">
+        <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>27.439</v>
+        <v>29.143</v>
       </c>
       <c r="U3" t="n">
         <v>2</v>
@@ -5150,75 +5091,73 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>DRREDDY</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>TTM</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>17.45</v>
-      </c>
-      <c r="D4" t="n">
-        <v>26.61</v>
-      </c>
-      <c r="E4" t="n">
-        <v>19.74</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="G4" t="n">
-        <v>33.24</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="I4" t="n">
-        <v>8577</v>
-      </c>
-      <c r="J4" t="n">
-        <v>4034</v>
-      </c>
-      <c r="K4" t="n">
-        <v>64</v>
-      </c>
-      <c r="L4" t="n">
-        <v>12</v>
-      </c>
-      <c r="M4" t="n">
-        <v>2002</v>
-      </c>
-      <c r="N4" t="n">
-        <v>4543</v>
-      </c>
-      <c r="O4" t="n">
-        <v>8.42</v>
-      </c>
-      <c r="P4" t="n">
-        <v>11.18</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>11.15</v>
-      </c>
-      <c r="R4" t="inlineStr">
+      <c r="C4" s="3" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>27.95</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>15.09</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>65.40000000000001</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>12898</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>763</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>3274</v>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>12135</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>48.73</v>
+      </c>
+      <c r="Q4" s="3" t="n">
+        <v>39.92</v>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>Pharmaceuticals</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T4" t="n">
-        <v>20.677</v>
-      </c>
-      <c r="U4" t="n">
+      <c r="S4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="T4" s="3" t="n">
+        <v>27.614</v>
+      </c>
+      <c r="U4" s="3" t="n">
         <v>3</v>
       </c>
       <c r="V4" s="2" t="n">
@@ -5228,7 +5167,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -5237,62 +5176,60 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>22.1</v>
+        <v>17.45</v>
       </c>
       <c r="D5" t="n">
-        <v>27.95</v>
+        <v>26.61</v>
       </c>
       <c r="E5" t="n">
-        <v>15.09</v>
+        <v>19.74</v>
       </c>
       <c r="F5" t="n">
-        <v>0.05</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>65.40000000000001</v>
+        <v>33.24</v>
       </c>
       <c r="H5" t="n">
-        <v>0.57</v>
+        <v>0.72</v>
       </c>
       <c r="I5" t="n">
-        <v>12898</v>
+        <v>8577</v>
       </c>
       <c r="J5" t="n">
-        <v>763</v>
+        <v>4034</v>
       </c>
       <c r="K5" t="n">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="L5" t="n">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="M5" t="n">
-        <v>3274</v>
+        <v>2002</v>
       </c>
       <c r="N5" t="n">
-        <v>12135</v>
+        <v>4543</v>
       </c>
       <c r="O5" t="n">
-        <v>13.39</v>
+        <v>13.16</v>
       </c>
       <c r="P5" t="n">
-        <v>10.19</v>
+        <v>29.25</v>
       </c>
       <c r="Q5" t="n">
-        <v>10.42</v>
+        <v>29.16</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
           <t>Pharmaceuticals</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="S5" t="n">
+        <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>20.444</v>
+        <v>25.239</v>
       </c>
       <c r="U5" t="n">
         <v>4</v>
@@ -5349,31 +5286,29 @@
         <v>3266</v>
       </c>
       <c r="O6" t="n">
-        <v>11.08</v>
+        <v>9.01</v>
       </c>
       <c r="P6" t="n">
-        <v>12.88</v>
+        <v>10.43</v>
       </c>
       <c r="Q6" t="n">
-        <v>12.77</v>
+        <v>10.42</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
           <t>Pharmaceuticals</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S6" t="n">
+        <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>19.308</v>
+        <v>18.404</v>
       </c>
       <c r="U6" t="n">
         <v>5</v>
       </c>
-      <c r="V6" s="3" t="n">
+      <c r="V6" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -5421,18 +5356,20 @@
         <v>4134</v>
       </c>
       <c r="O7" t="n">
-        <v>11.08</v>
+        <v>9.01</v>
       </c>
       <c r="P7" t="n">
-        <v>10.26</v>
+        <v>20.2</v>
       </c>
       <c r="Q7" t="n">
-        <v>10.42</v>
+        <v>19.9</v>
       </c>
       <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
       <c r="T7" t="n">
-        <v>20.677</v>
+        <v>27.614</v>
       </c>
       <c r="U7" t="n">
         <v>3</v>
@@ -5570,7 +5507,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>ADANIGREEN</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5579,62 +5516,60 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>34.3</v>
+        <v>17.88</v>
       </c>
       <c r="D2" t="n">
-        <v>85.64</v>
+        <v>75.13</v>
       </c>
       <c r="E2" t="n">
-        <v>17.87</v>
+        <v>12.81</v>
       </c>
       <c r="F2" t="n">
-        <v>1.42</v>
+        <v>6.6</v>
       </c>
       <c r="G2" t="n">
-        <v>4.64</v>
+        <v>1.81</v>
       </c>
       <c r="H2" t="n">
-        <v>0.18</v>
+        <v>0.1</v>
       </c>
       <c r="I2" t="n">
-        <v>50404</v>
+        <v>28773</v>
       </c>
       <c r="J2" t="n">
-        <v>13114</v>
+        <v>21060</v>
       </c>
       <c r="K2" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="L2" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>123516</v>
+        <v>64858</v>
       </c>
       <c r="N2" t="n">
-        <v>37290</v>
+        <v>7713</v>
       </c>
       <c r="O2" t="n">
-        <v>11.01</v>
+        <v>36.3</v>
       </c>
       <c r="P2" t="n">
-        <v>11.37</v>
+        <v>80.41</v>
       </c>
       <c r="Q2" t="n">
-        <v>10.74</v>
+        <v>73.20999999999999</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
           <t>Power &amp; Utilities</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S2" t="n">
+        <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>27.67100000000001</v>
+        <v>43.23</v>
       </c>
       <c r="U2" t="n">
         <v>1</v>
@@ -5646,7 +5581,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TATAPOWER</t>
+          <t>ADANIPOWER</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5655,72 +5590,72 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>6.94</v>
+        <v>23.21</v>
       </c>
       <c r="D3" t="n">
-        <v>17.42</v>
+        <v>38.36</v>
       </c>
       <c r="E3" t="n">
-        <v>13.23</v>
+        <v>48.28</v>
       </c>
       <c r="F3" t="n">
-        <v>1.66</v>
+        <v>0.8</v>
       </c>
       <c r="G3" t="n">
-        <v>3.25</v>
+        <v>7.14</v>
       </c>
       <c r="H3" t="n">
-        <v>0.44</v>
+        <v>0.55</v>
       </c>
       <c r="I3" t="n">
-        <v>21623</v>
+        <v>17651</v>
       </c>
       <c r="J3" t="n">
-        <v>9027</v>
+        <v>3481</v>
       </c>
       <c r="K3" t="n">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="L3" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>53689</v>
+        <v>34616</v>
       </c>
       <c r="N3" t="n">
-        <v>12596</v>
+        <v>14170</v>
       </c>
       <c r="O3" t="n">
-        <v>5.56</v>
+        <v>20.15</v>
       </c>
       <c r="P3" t="n">
-        <v>34.74</v>
-      </c>
-      <c r="Q3" t="inlineStr"/>
+        <v>77.78</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>82.12</v>
+      </c>
       <c r="R3" t="inlineStr">
         <is>
           <t>Power &amp; Utilities</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S3" t="n">
+        <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>15.828</v>
+        <v>42.14</v>
       </c>
       <c r="U3" t="n">
         <v>2</v>
       </c>
       <c r="V3" s="1" t="n">
-        <v>80</v>
+        <v>85.70999999999999</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NHPC</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -5729,68 +5664,66 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>35.26</v>
+        <v>34.3</v>
       </c>
       <c r="D4" t="n">
-        <v>51.75</v>
+        <v>85.64</v>
       </c>
       <c r="E4" t="n">
-        <v>10.41</v>
+        <v>17.87</v>
       </c>
       <c r="F4" t="n">
-        <v>0.84</v>
+        <v>1.42</v>
       </c>
       <c r="G4" t="n">
-        <v>9.9</v>
+        <v>4.64</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1</v>
+        <v>0.18</v>
       </c>
       <c r="I4" t="n">
-        <v>12906</v>
+        <v>50404</v>
       </c>
       <c r="J4" t="n">
-        <v>5968</v>
+        <v>13114</v>
       </c>
       <c r="K4" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="L4" t="n">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="M4" t="n">
-        <v>32561</v>
+        <v>123516</v>
       </c>
       <c r="N4" t="n">
-        <v>6938</v>
+        <v>37290</v>
       </c>
       <c r="O4" t="n">
-        <v>3.54</v>
+        <v>3.68</v>
       </c>
       <c r="P4" t="n">
-        <v>1.46</v>
+        <v>6.89</v>
       </c>
       <c r="Q4" t="n">
-        <v>3.44</v>
+        <v>6.94</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
           <t>Power &amp; Utilities</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S4" t="n">
+        <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>15.229</v>
+        <v>25.309</v>
       </c>
       <c r="U4" t="n">
         <v>3</v>
       </c>
       <c r="V4" s="2" t="n">
-        <v>60</v>
+        <v>71.43000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -5841,38 +5774,36 @@
         <v>6234</v>
       </c>
       <c r="O5" t="n">
-        <v>2.13</v>
+        <v>13.32</v>
       </c>
       <c r="P5" t="n">
-        <v>6.82</v>
+        <v>24.67</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.18</v>
+        <v>21.79</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
           <t>Power &amp; Utilities</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S5" t="n">
+        <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>13.931</v>
+        <v>19.739</v>
       </c>
       <c r="U5" t="n">
         <v>4</v>
       </c>
       <c r="V5" s="2" t="n">
-        <v>40</v>
+        <v>57.14</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>TATAPOWER</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -5881,140 +5812,146 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>12.13</v>
+        <v>6.94</v>
       </c>
       <c r="D6" t="n">
-        <v>28.18</v>
+        <v>17.42</v>
       </c>
       <c r="E6" t="n">
-        <v>13.27</v>
+        <v>13.23</v>
       </c>
       <c r="F6" t="n">
-        <v>1.48</v>
+        <v>1.66</v>
       </c>
       <c r="G6" t="n">
-        <v>4.75</v>
+        <v>3.25</v>
       </c>
       <c r="H6" t="n">
-        <v>0.37</v>
+        <v>0.44</v>
       </c>
       <c r="I6" t="n">
-        <v>72926</v>
+        <v>21623</v>
       </c>
       <c r="J6" t="n">
-        <v>32141</v>
+        <v>9027</v>
       </c>
       <c r="K6" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="L6" t="n">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="M6" t="n">
-        <v>237131</v>
+        <v>53689</v>
       </c>
       <c r="N6" t="n">
-        <v>40785</v>
+        <v>12596</v>
       </c>
       <c r="O6" t="n">
-        <v>8.289999999999999</v>
+        <v>18.04</v>
       </c>
       <c r="P6" t="n">
-        <v>4.98</v>
+        <v>32.26</v>
       </c>
       <c r="Q6" t="n">
-        <v>4.87</v>
+        <v>31.61</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
           <t>Power &amp; Utilities</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="S6" t="n">
+        <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>12.861</v>
+        <v>17.828</v>
       </c>
       <c r="U6" t="n">
         <v>5</v>
       </c>
-      <c r="V6" s="3" t="n">
-        <v>20</v>
+      <c r="V6" s="2" t="n">
+        <v>42.86</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>ADANIGREEN</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>TTM</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>17.88</v>
-      </c>
-      <c r="D7" t="n">
-        <v>75.13</v>
-      </c>
-      <c r="E7" t="n">
-        <v>12.81</v>
-      </c>
-      <c r="F7" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="G7" t="n">
-        <v>1.81</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I7" t="n">
-        <v>28773</v>
-      </c>
-      <c r="J7" t="n">
-        <v>21060</v>
-      </c>
-      <c r="K7" t="n">
-        <v>9</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" t="n">
-        <v>64858</v>
-      </c>
-      <c r="N7" t="n">
-        <v>7713</v>
-      </c>
-      <c r="O7" t="n">
-        <v>46.72</v>
-      </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr">
+      <c r="C7" s="3" t="n">
+        <v>12.13</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>28.18</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>13.27</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>72926</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>32141</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="L7" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="M7" s="3" t="n">
+        <v>237131</v>
+      </c>
+      <c r="N7" s="3" t="n">
+        <v>40785</v>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>13.62</v>
+      </c>
+      <c r="P7" s="3" t="n">
+        <v>10.78</v>
+      </c>
+      <c r="Q7" s="3" t="n">
+        <v>11.28</v>
+      </c>
+      <c r="R7" s="3" t="inlineStr">
         <is>
           <t>Power &amp; Utilities</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
+      <c r="S7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="T7" s="3" t="n">
+        <v>15.087</v>
+      </c>
+      <c r="U7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="V7" s="2" t="n">
+        <v>28.57</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ADANIPOWER</t>
+          <t>NHPC</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6023,59 +5960,67 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>23.21</v>
+        <v>35.26</v>
       </c>
       <c r="D8" t="n">
-        <v>38.36</v>
+        <v>51.75</v>
       </c>
       <c r="E8" t="n">
-        <v>48.28</v>
+        <v>10.41</v>
       </c>
       <c r="F8" t="n">
-        <v>0.8</v>
+        <v>0.84</v>
       </c>
       <c r="G8" t="n">
-        <v>7.14</v>
+        <v>9.9</v>
       </c>
       <c r="H8" t="n">
-        <v>0.55</v>
+        <v>0.1</v>
       </c>
       <c r="I8" t="n">
-        <v>17651</v>
+        <v>12906</v>
       </c>
       <c r="J8" t="n">
-        <v>3481</v>
+        <v>5968</v>
       </c>
       <c r="K8" t="n">
-        <v>33</v>
+        <v>3</v>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="M8" t="n">
-        <v>34616</v>
+        <v>32561</v>
       </c>
       <c r="N8" t="n">
-        <v>14170</v>
+        <v>6938</v>
       </c>
       <c r="O8" t="n">
-        <v>19.12</v>
-      </c>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
+        <v>0.11</v>
+      </c>
+      <c r="P8" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
       <c r="R8" t="inlineStr">
         <is>
           <t>Power &amp; Utilities</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
+      <c r="S8" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" t="n">
+        <v>13.991</v>
+      </c>
+      <c r="U8" t="n">
+        <v>7</v>
+      </c>
+      <c r="V8" s="4" t="n">
+        <v>14.29</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -6121,24 +6066,26 @@
         <v>12596</v>
       </c>
       <c r="O9" t="n">
-        <v>8.289999999999999</v>
+        <v>13.62</v>
       </c>
       <c r="P9" t="n">
-        <v>6.82</v>
+        <v>24.67</v>
       </c>
       <c r="Q9" t="n">
-        <v>5.025</v>
+        <v>21.79</v>
       </c>
       <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
+      <c r="S9" t="n">
+        <v>0</v>
+      </c>
       <c r="T9" t="n">
-        <v>15.229</v>
+        <v>19.739</v>
       </c>
       <c r="U9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V9" s="2" t="n">
-        <v>60</v>
+        <v>57.14</v>
       </c>
     </row>
   </sheetData>
@@ -6315,26 +6262,24 @@
         <v>15685</v>
       </c>
       <c r="O2" t="n">
-        <v>15.96</v>
+        <v>18.2</v>
       </c>
       <c r="P2" t="n">
-        <v>21.22</v>
+        <v>22.55</v>
       </c>
       <c r="Q2" t="n">
-        <v>18.33</v>
+        <v>22.61</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
           <t>Private Banks</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S2" t="n">
+        <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>28.497</v>
+        <v>29.211</v>
       </c>
       <c r="U2" t="n">
         <v>1</v>
@@ -6346,7 +6291,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6355,62 +6300,60 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>21.93</v>
+        <v>29.03</v>
       </c>
       <c r="D3" t="n">
-        <v>62.61</v>
+        <v>69.63</v>
       </c>
       <c r="E3" t="n">
-        <v>14.34</v>
+        <v>17.99</v>
       </c>
       <c r="F3" t="n">
-        <v>6.81</v>
+        <v>6.45</v>
       </c>
       <c r="G3" t="n">
-        <v>1.41</v>
+        <v>1.23</v>
       </c>
       <c r="H3" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>35669</v>
+        <v>302021</v>
       </c>
       <c r="J3" t="n">
-        <v>16600</v>
+        <v>144737</v>
       </c>
       <c r="K3" t="n">
-        <v>91</v>
+        <v>70</v>
       </c>
       <c r="L3" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="M3" t="n">
-        <v>3107503</v>
+        <v>1651008</v>
       </c>
       <c r="N3" t="n">
-        <v>19069</v>
+        <v>157284</v>
       </c>
       <c r="O3" t="n">
-        <v>20.29</v>
+        <v>19.29</v>
       </c>
       <c r="P3" t="n">
-        <v>21.6</v>
+        <v>26.66</v>
       </c>
       <c r="Q3" t="n">
-        <v>16.88</v>
+        <v>26.89</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
           <t>Private Banks</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="S3" t="n">
+        <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>25.102</v>
+        <v>27.199</v>
       </c>
       <c r="U3" t="n">
         <v>2</v>
@@ -6420,75 +6363,73 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>ICICIBANK</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>TTM</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>29.03</v>
-      </c>
-      <c r="D4" t="n">
-        <v>69.63</v>
-      </c>
-      <c r="E4" t="n">
-        <v>17.99</v>
-      </c>
-      <c r="F4" t="n">
-        <v>6.45</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1.23</v>
-      </c>
-      <c r="H4" t="n">
+      <c r="C4" s="3" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>62.61</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>14.34</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>6.81</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="H4" s="3" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="I4" t="n">
-        <v>302021</v>
-      </c>
-      <c r="J4" t="n">
-        <v>144737</v>
-      </c>
-      <c r="K4" t="n">
-        <v>70</v>
-      </c>
-      <c r="L4" t="n">
-        <v>16</v>
-      </c>
-      <c r="M4" t="n">
-        <v>1651008</v>
-      </c>
-      <c r="N4" t="n">
-        <v>157284</v>
-      </c>
-      <c r="O4" t="n">
-        <v>12.3</v>
-      </c>
-      <c r="P4" t="n">
-        <v>14.68</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>13.7</v>
-      </c>
-      <c r="R4" t="inlineStr">
+      <c r="I4" s="3" t="n">
+        <v>35669</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>16600</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>91</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>3107503</v>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>19069</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>26.48</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>22.68</v>
+      </c>
+      <c r="Q4" s="3" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>Private Banks</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T4" t="n">
-        <v>23.405</v>
-      </c>
-      <c r="U4" t="n">
+      <c r="S4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="T4" s="3" t="n">
+        <v>26.556</v>
+      </c>
+      <c r="U4" s="3" t="n">
         <v>3</v>
       </c>
       <c r="V4" s="2" t="n">
@@ -6498,7 +6439,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>INDUSINDBK</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6507,62 +6448,60 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>16.57</v>
+        <v>21.87</v>
       </c>
       <c r="D5" t="n">
-        <v>41.03</v>
+        <v>36.94</v>
       </c>
       <c r="E5" t="n">
-        <v>14.25</v>
+        <v>15.83</v>
       </c>
       <c r="F5" t="n">
-        <v>6.89</v>
+        <v>8.25</v>
       </c>
       <c r="G5" t="n">
-        <v>2.11</v>
+        <v>1.77</v>
       </c>
       <c r="H5" t="n">
-        <v>0.09</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="I5" t="n">
-        <v>-16218</v>
+        <v>3446</v>
       </c>
       <c r="J5" t="n">
-        <v>625</v>
+        <v>9001</v>
       </c>
       <c r="K5" t="n">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="L5" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="M5" t="n">
-        <v>432404</v>
+        <v>1295302</v>
       </c>
       <c r="N5" t="n">
-        <v>-16843</v>
+        <v>-5555</v>
       </c>
       <c r="O5" t="n">
-        <v>17.63</v>
+        <v>17.48</v>
       </c>
       <c r="P5" t="n">
-        <v>18.48</v>
+        <v>41.47</v>
       </c>
       <c r="Q5" t="n">
-        <v>14.73</v>
+        <v>40.2</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
           <t>Private Banks</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S5" t="n">
+        <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>19.395</v>
+        <v>23.646</v>
       </c>
       <c r="U5" t="n">
         <v>4</v>
@@ -6574,7 +6513,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>INDUSINDBK</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6583,67 +6522,65 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>21.87</v>
+        <v>16.57</v>
       </c>
       <c r="D6" t="n">
-        <v>36.94</v>
+        <v>41.03</v>
       </c>
       <c r="E6" t="n">
-        <v>15.83</v>
+        <v>14.25</v>
       </c>
       <c r="F6" t="n">
-        <v>8.25</v>
+        <v>6.89</v>
       </c>
       <c r="G6" t="n">
-        <v>1.77</v>
+        <v>2.11</v>
       </c>
       <c r="H6" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.09</v>
       </c>
       <c r="I6" t="n">
-        <v>3446</v>
+        <v>-16218</v>
       </c>
       <c r="J6" t="n">
-        <v>9001</v>
+        <v>625</v>
       </c>
       <c r="K6" t="n">
-        <v>85</v>
+        <v>104</v>
       </c>
       <c r="L6" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="M6" t="n">
-        <v>1295302</v>
+        <v>432404</v>
       </c>
       <c r="N6" t="n">
-        <v>-5555</v>
+        <v>-16843</v>
       </c>
       <c r="O6" t="n">
-        <v>13.22</v>
+        <v>14.01</v>
       </c>
       <c r="P6" t="n">
-        <v>14.53</v>
+        <v>30.09</v>
       </c>
       <c r="Q6" t="n">
-        <v>11.92</v>
+        <v>29.48</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
           <t>Private Banks</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="S6" t="n">
+        <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>17.406</v>
+        <v>20.993</v>
       </c>
       <c r="U6" t="n">
         <v>5</v>
       </c>
-      <c r="V6" s="3" t="n">
+      <c r="V6" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -6691,18 +6628,20 @@
         <v>15685</v>
       </c>
       <c r="O7" t="n">
-        <v>15.96</v>
+        <v>18.2</v>
       </c>
       <c r="P7" t="n">
-        <v>18.48</v>
+        <v>26.66</v>
       </c>
       <c r="Q7" t="n">
-        <v>14.73</v>
+        <v>26.89</v>
       </c>
       <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
       <c r="T7" t="n">
-        <v>23.405</v>
+        <v>26.556</v>
       </c>
       <c r="U7" t="n">
         <v>3</v>

</xml_diff>